<commit_message>
Fix P13 worksheet ordering and record native Excel opening proof
</commit_message>
<xml_diff>
--- a/tools/candidates/remaining-batch-r3-20261018/checkpoint-working/P13/63-reestr-zatrat-po-obektu.xlsx
+++ b/tools/candidates/remaining-batch-r3-20261018/checkpoint-working/P13/63-reestr-zatrat-po-obektu.xlsx
@@ -1751,35 +1751,35 @@
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="10" t="inlineStr"/>
     </row>
-    <row r="54">
-      <c r="C54" t="str" s="14">
-        <v>Предварительно не покрыто ценой:</v>
-      </c>
-      <c r="H54" t="n" s="12">
-        <f>SUMIFS(H2:H52,I2:I52,"&lt;&gt;покрыто, проверено",I2:I52,"&lt;&gt;принято",I2:I52,"&lt;&gt;не применяется")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" t="inlineStr" s="15">
-        <is>
-          <t>Плановая прибыль по объекту:</t>
-        </is>
-      </c>
-      <c r="H55" s="11" t="n"/>
-    </row>
-    <row r="56">
-      <c r="C56" t="str" s="15">
-        <v>Непокрытая сумма / плановая прибыль:</v>
-      </c>
-      <c r="H56" t="str" s="13">
-        <f>IF(OR(H55="",H55&lt;=0),"",H54/H55)</f>
-      </c>
-    </row>
     <row r="53" ht="22" customHeight="1">
       <c r="C53" t="str" s="15">
         <f>IF(COUNTBLANK(D2:D52)&gt;0,"Заполните покрытие всех 51 строк; неприменимые отметьте явно",IF(COUNTBLANK(I2:I52)&gt;0,"Заполните статус каждой строки",IF(SUMPRODUCT((I2:I52&lt;&gt;"покрыто, проверено")*(I2:I52&lt;&gt;"принято")*(I2:I52&lt;&gt;"не применяется")*(ISNUMBER(H2:H52)=FALSE))&gt;0,"Есть непокрытые затраты без числовой оценки",IF(SUMPRODUCT(((I2:I52="покрыто, проверено")+(I2:I52="принято"))*(G2:G52=""))&gt;0,"Укажите документы покрытия для закрытых позиций","Проверка заполнена; решение о цене принимает руководитель"))))</f>
         <v>Заполните покрытие всех 51 строк; неприменимые отметьте явно</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="str" s="14">
+        <v>Предварительно не покрыто ценой:</v>
+      </c>
+      <c r="H54" t="n" s="12">
+        <f>SUMIFS(H2:H52,I2:I52,"&lt;&gt;покрыто, проверено",I2:I52,"&lt;&gt;принято",I2:I52,"&lt;&gt;не применяется")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" t="inlineStr" s="15">
+        <is>
+          <t>Плановая прибыль по объекту:</t>
+        </is>
+      </c>
+      <c r="H55" s="11" t="n"/>
+    </row>
+    <row r="56">
+      <c r="C56" t="str" s="15">
+        <v>Непокрытая сумма / плановая прибыль:</v>
+      </c>
+      <c r="H56" t="str" s="13">
+        <f>IF(OR(H55="",H55&lt;=0),"",H54/H55)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>